<commit_message>
Further updates to templates
</commit_message>
<xml_diff>
--- a/src/templates/pricing_spreadsheet.xlsx
+++ b/src/templates/pricing_spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joseph\Desktop\Code\MSSProposalAutomation\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99567BE3-290F-49F4-828B-B7BBA1332BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A9B45B-0389-4424-9CCD-1A78EE6ED479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="1" xr2:uid="{25869D54-3781-4886-8FF9-0A7E0B41E358}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="219">
   <si>
     <t>AC Breaker</t>
   </si>
@@ -684,6 +684,21 @@
   </si>
   <si>
     <t>{{PANEL_COUNT}}</t>
+  </si>
+  <si>
+    <t>Utility</t>
+  </si>
+  <si>
+    <t>Tree Trimming Required?</t>
+  </si>
+  <si>
+    <t>Loan Term</t>
+  </si>
+  <si>
+    <t>Interest Rate</t>
+  </si>
+  <si>
+    <t>Monthly Payment</t>
   </si>
 </sst>
 </file>
@@ -1061,7 +1076,7 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="27" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="180">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1428,6 +1443,13 @@
     </xf>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="1" xfId="18" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="18" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1436,6 +1458,16 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="10" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="14" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="20">
@@ -3201,6 +3233,23 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -3568,8 +3617,9 @@
         <v>156</v>
       </c>
       <c r="B10" s="82"/>
-      <c r="C10" s="5" t="s">
-        <v>73</v>
+      <c r="C10" s="5" t="str">
+        <f>'Edit Variables'!B2</f>
+        <v>MID</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -3618,7 +3668,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1710F80-8E9B-42D2-B4C6-C5445B098A6C}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="12.45"/>
   <cols>
     <col min="1" max="1" width="40.69140625" customWidth="1"/>
@@ -3633,12 +3683,33 @@
         <v>211</v>
       </c>
     </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" s="172" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>A1=""</formula>
+      <formula>B1=""</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{60B8E31B-39B7-4944-9BC6-9AF1B77C6E94}">
+      <formula1>"MID, PG&amp;E"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5391,12 +5462,44 @@
       <c r="I107" s="171"/>
     </row>
     <row r="108" spans="1:12">
+      <c r="C108" s="158" t="s">
+        <v>216</v>
+      </c>
+      <c r="D108" s="176">
+        <v>12</v>
+      </c>
       <c r="K108" s="171"/>
     </row>
     <row r="109" spans="1:12">
-      <c r="C109" s="158"/>
-    </row>
-    <row r="125" spans="9:9">
+      <c r="C109" s="158" t="s">
+        <v>217</v>
+      </c>
+      <c r="D109" s="178">
+        <v>6.7400000000000002E-2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12">
+      <c r="C110" s="177" t="s">
+        <v>218</v>
+      </c>
+      <c r="D110" s="179">
+        <f>D88*(((D109/12)*(1+(D109/12))^(D108*12))/(((1+(D109/12))^(D108*12))-1))</f>
+        <v>343.73752351267893</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12">
+      <c r="C111" s="158"/>
+      <c r="D111" s="158"/>
+    </row>
+    <row r="112" spans="1:12">
+      <c r="C112" s="158"/>
+      <c r="D112" s="158"/>
+    </row>
+    <row r="113" spans="3:9">
+      <c r="C113" s="158"/>
+      <c r="D113" s="158"/>
+    </row>
+    <row r="125" spans="3:9">
       <c r="I125" s="5" t="s">
         <v>107</v>
       </c>
@@ -6056,11 +6159,11 @@
       </c>
       <c r="G26" s="52"/>
       <c r="H26" s="52"/>
-      <c r="K26" s="172" t="s">
+      <c r="K26" s="173" t="s">
         <v>181</v>
       </c>
-      <c r="L26" s="172"/>
-      <c r="M26" s="172"/>
+      <c r="L26" s="173"/>
+      <c r="M26" s="173"/>
     </row>
     <row r="27" spans="1:24" ht="12.9">
       <c r="A27"/>
@@ -6791,26 +6894,26 @@
       </c>
     </row>
     <row r="15" spans="1:10">
-      <c r="B15" s="173" t="s">
+      <c r="B15" s="174" t="s">
         <v>123</v>
       </c>
-      <c r="C15" s="173"/>
-      <c r="D15" s="173"/>
-      <c r="G15" s="173" t="s">
+      <c r="C15" s="174"/>
+      <c r="D15" s="174"/>
+      <c r="G15" s="174" t="s">
         <v>122</v>
       </c>
-      <c r="H15" s="173"/>
-      <c r="I15" s="173"/>
-      <c r="J15" s="173"/>
+      <c r="H15" s="174"/>
+      <c r="I15" s="174"/>
+      <c r="J15" s="174"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="B17" s="174" t="s">
+      <c r="B17" s="175" t="s">
         <v>127</v>
       </c>
-      <c r="C17" s="174" t="s">
+      <c r="C17" s="175" t="s">
         <v>128</v>
       </c>
-      <c r="D17" s="174" t="s">
+      <c r="D17" s="175" t="s">
         <v>129</v>
       </c>
       <c r="G17" s="63" t="s">
@@ -6827,9 +6930,9 @@
       </c>
     </row>
     <row r="18" spans="1:10">
-      <c r="B18" s="174"/>
-      <c r="C18" s="174"/>
-      <c r="D18" s="174"/>
+      <c r="B18" s="175"/>
+      <c r="C18" s="175"/>
+      <c r="D18" s="175"/>
       <c r="F18" t="str">
         <f>H9</f>
         <v>{{YEAR}}</v>

</xml_diff>